<commit_message>
updating backtesting system for final prototype...
</commit_message>
<xml_diff>
--- a/automated_backtesting_results/full_backtesting_tables_excel/final_backtesting_summary_AAPL.xlsx
+++ b/automated_backtesting_results/full_backtesting_tables_excel/final_backtesting_summary_AAPL.xlsx
@@ -469,10 +469,10 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="19" customWidth="1" min="12" max="12"/>
     <col width="23" customWidth="1" min="13" max="13"/>
@@ -524,7 +524,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>CAGR Efficiency</t>
+          <t>CAGR Efficiency (%)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -539,7 +539,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Sharpe Efficiency</t>
+          <t>Sharpe Efficiency (%)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -656,7 +656,7 @@
         <v>0.49</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-0.68</v>
+        <v>-68.16</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>-0.42</v>

</xml_diff>